<commit_message>
fixed the db when the app is packaged
</commit_message>
<xml_diff>
--- a/data/new_data.xlsx
+++ b/data/new_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
@@ -4880,6 +4880,16 @@
       </c>
     </row>
     <row r="34" customFormat="1" s="55">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NOVOCIB Rapport d'essai 260722-2.docx</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>260722-2</t>
+        </is>
+      </c>
       <c r="C34" s="56" t="n">
         <v>2</v>
       </c>
@@ -6224,7 +6234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.140625" customWidth="1" min="1" max="1"/>
@@ -6243,6 +6253,16 @@
           <t>Critere</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>numero rapport</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>nom rapport generé</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -6342,6 +6362,28 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>260722-3</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>NOVOCIB Rapport d'essai 260722-3.docx</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>260722-3</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NOVOCIB Rapport d'essai 260722-3.docx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
re-fixed the file name when saving & excel not selecting the correct sheet
</commit_message>
<xml_diff>
--- a/data/new_data.xlsx
+++ b/data/new_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
@@ -4762,6 +4762,16 @@
       <c r="AD32" s="22" t="n"/>
     </row>
     <row r="33" customFormat="1" s="55">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NOVOCIB Rapport d'essai 260722-1.docx</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>260722-1</t>
+        </is>
+      </c>
       <c r="C33" s="56" t="n">
         <v>1</v>
       </c>
@@ -4880,16 +4890,6 @@
       </c>
     </row>
     <row r="34" customFormat="1" s="55">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>NOVOCIB Rapport d'essai 260722-2.docx</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>260722-2</t>
-        </is>
-      </c>
       <c r="C34" s="56" t="n">
         <v>2</v>
       </c>
@@ -5008,16 +5008,6 @@
       </c>
     </row>
     <row r="35" customFormat="1" s="55">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>NOVOCIB Rapport d'essai 260722-3.docx</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>260722-3</t>
-        </is>
-      </c>
       <c r="C35" s="56" t="n">
         <v>3</v>
       </c>
@@ -6234,7 +6224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.140625" customWidth="1" min="1" max="1"/>
@@ -6253,16 +6243,6 @@
           <t>Critere</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>numero rapport</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>nom rapport generé</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -6362,28 +6342,6 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>260722-3</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>NOVOCIB Rapport d'essai 260722-3.docx</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>260722-3</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>NOVOCIB Rapport d'essai 260722-3.docx</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>